<commit_message>
ramping angepasst und h2-kaverne erweitert. grafische auswertung akutalisiert
</commit_message>
<xml_diff>
--- a/data/a_Eingangsdaten/Optimierungsgrößen - mit Speicher_Strom.xlsx
+++ b/data/a_Eingangsdaten/Optimierungsgrößen - mit Speicher_Strom.xlsx
@@ -713,11 +713,11 @@
       <c r="D10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="1" t="n">
-        <v>47000</v>
+      <c r="E10" s="0" t="n">
+        <v>2000000</v>
       </c>
       <c r="F10" s="1" t="n">
-        <v>1868.5</v>
+        <v>1870.5</v>
       </c>
       <c r="G10" s="1" t="n">
         <v>0.4</v>
@@ -725,8 +725,8 @@
       <c r="H10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="1" t="n">
-        <v>33000000</v>
+      <c r="I10" s="0" t="n">
+        <v>1600000000</v>
       </c>
       <c r="J10" s="1" t="n">
         <v>0.001</v>

</xml_diff>

<commit_message>
Auswertung zunächst in excel
</commit_message>
<xml_diff>
--- a/data/a_Eingangsdaten/Optimierungsgrößen - mit Speicher_Strom.xlsx
+++ b/data/a_Eingangsdaten/Optimierungsgrößen - mit Speicher_Strom.xlsx
@@ -382,7 +382,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="17.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="24.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="13.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="29.63"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -691,7 +691,7 @@
         <v>60666</v>
       </c>
       <c r="I9" s="1" t="n">
-        <v>304300000</v>
+        <v>304300</v>
       </c>
       <c r="J9" s="1" t="n">
         <v>0.001</v>
@@ -713,7 +713,7 @@
       <c r="D10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="0" t="n">
+      <c r="E10" s="1" t="n">
         <v>2000000</v>
       </c>
       <c r="F10" s="1" t="n">
@@ -725,7 +725,7 @@
       <c r="H10" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="I10" s="0" t="n">
+      <c r="I10" s="1" t="n">
         <v>1600000000</v>
       </c>
       <c r="J10" s="1" t="n">

</xml_diff>